<commit_message>
updates to correct errors in land cover look up table
</commit_message>
<xml_diff>
--- a/Neltuma_Mlr3_Pipeline/data_in/Veg_type_lookup_list.xlsx
+++ b/Neltuma_Mlr3_Pipeline/data_in/Veg_type_lookup_list.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Botswana_Research\QField\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Slade_et_al_mapping_invasive_Neltuma_Kalahari\Neltuma_Mlr3_Pipeline\data_in\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD2D988-48A7-48E2-A74E-6501978215F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11490" windowHeight="4980"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,44 +25,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
-  <si>
-    <t>Prosopis</t>
-  </si>
-  <si>
-    <t>Bare Sand</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Short Grass</t>
   </si>
   <si>
-    <t>Gnidia</t>
-  </si>
-  <si>
-    <t>Camel Thorn</t>
-  </si>
-  <si>
-    <t>Rig Trig</t>
-  </si>
-  <si>
-    <t>Acacia Melifera</t>
-  </si>
-  <si>
     <t>Calcrete</t>
   </si>
   <si>
-    <t>Blue Bush</t>
-  </si>
-  <si>
-    <t>Shepherds Tree</t>
-  </si>
-  <si>
     <t>Other- record in notes</t>
   </si>
   <si>
-    <t>Candle Bush</t>
-  </si>
-  <si>
     <t>Tall Dune Grass</t>
   </si>
   <si>
@@ -74,9 +48,6 @@
     <t>White exposed limestone rock</t>
   </si>
   <si>
-    <t>Tall (3-7m)Tree mostly still green in dry season - some (c.50% ) flowering with small orange flowers</t>
-  </si>
-  <si>
     <t>Low (c.1m) Blueish grey shrub</t>
   </si>
   <si>
@@ -89,25 +60,64 @@
     <t>Mostly light brown/orange coloured bare sand</t>
   </si>
   <si>
-    <t xml:space="preserve">Dry grey/brown grass (&lt;0.5m)with associated leaf litter </t>
-  </si>
-  <si>
     <t>Tall 2-4m Tree - dark green leaves - rare individuals</t>
   </si>
   <si>
     <t>Low (c.1 - 1.5 m) Bush often circular in shape</t>
   </si>
   <si>
-    <t>Light brown/grey Grass - thick clumps (c.1m) in height</t>
-  </si>
-  <si>
     <t>Individual trees such as Acacia Haematoxylon - not used in classification as too rare to use for training and validation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dry grey/brown grass (&lt; 0.5 m) with associated leaf litter </t>
+  </si>
+  <si>
+    <t>Class_Number</t>
+  </si>
+  <si>
+    <t>Class_Name</t>
+  </si>
+  <si>
+    <t>Class_Description</t>
+  </si>
+  <si>
+    <t>Neltuma</t>
+  </si>
+  <si>
+    <t>Bare Ground</t>
+  </si>
+  <si>
+    <t>Gnidia polycephala</t>
+  </si>
+  <si>
+    <t>Vachellia erioloba</t>
+  </si>
+  <si>
+    <t>Tall (3-7 m) Tree mostly still green in dry season - some (c.50% ) flowering with small orange flowers</t>
+  </si>
+  <si>
+    <t>Rhigozum trichotomum</t>
+  </si>
+  <si>
+    <t>Senegalia mellifera</t>
+  </si>
+  <si>
+    <t>Diospyros lycioides</t>
+  </si>
+  <si>
+    <t>Boscia albitrunca</t>
+  </si>
+  <si>
+    <t>Vachellia hebeclada</t>
+  </si>
+  <si>
+    <t>Light brown/grey Grass - thick clumps (c.1m) in height. Mostly Stipagrostis amabilis</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -137,8 +147,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,154 +431,165 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>11</v>
-      </c>
-      <c r="B11" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" t="s">
-        <v>24</v>
+      <c r="C14" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>